<commit_message>
Holiday home and cruise final project
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -3,21 +3,22 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coding\Hackathon_TripCost\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C66F9E5C-C83A-491A-B9BE-93A96B43E106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5650E13-2788-4FE8-B27B-B49005D99C77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{720C0748-C620-446B-B2C9-8C874C0E3B0F}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{720C0748-C620-446B-B2C9-8C874C0E3B0F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Cruises" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="75">
   <si>
     <t>TestCaseName</t>
   </si>
@@ -68,9 +69,6 @@
     <t>TC01</t>
   </si>
   <si>
-    <t>Elevator</t>
-  </si>
-  <si>
     <t>TC02</t>
   </si>
   <si>
@@ -89,9 +87,6 @@
     <t>Dubai</t>
   </si>
   <si>
-    <t>Swimming Pool</t>
-  </si>
-  <si>
     <t>5 stars</t>
   </si>
   <si>
@@ -101,9 +96,6 @@
     <t>Paris</t>
   </si>
   <si>
-    <t>Entire homes &amp; apts</t>
-  </si>
-  <si>
     <t>City view</t>
   </si>
   <si>
@@ -173,12 +165,6 @@
     <t>Bali</t>
   </si>
   <si>
-    <t>Private pool</t>
-  </si>
-  <si>
-    <t>Spa and wellness centre</t>
-  </si>
-  <si>
     <t>PASS</t>
   </si>
   <si>
@@ -218,9 +204,6 @@
     <t>11_testCase_blankDest</t>
   </si>
   <si>
-    <t>Free Wifi</t>
-  </si>
-  <si>
     <t>TC12</t>
   </si>
   <si>
@@ -243,13 +226,50 @@
   </si>
   <si>
     <t>@@@###$$$</t>
+  </si>
+  <si>
+    <t>Upper floors accessible by elevator</t>
+  </si>
+  <si>
+    <t>https://www.tripadvisor.com/Cruise_Review-d24948905-Reviews-Emerald_Cruises_Emerald_Luna</t>
+  </si>
+  <si>
+    <t>https://www.tripadvisor.com/Cruise_Review-d15611482-Reviews-Oasis_of_the_Seas</t>
+  </si>
+  <si>
+    <t>01_testCase_CruiseEmerald</t>
+  </si>
+  <si>
+    <t>02_testCase_CruiseOasis</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>Indoor pool</t>
+  </si>
+  <si>
+    <t>Spa</t>
+  </si>
+  <si>
+    <t>Top reviewed</t>
+  </si>
+  <si>
+    <t>Resorts</t>
+  </si>
+  <si>
+    <t>Breakfast &amp; dinner included</t>
+  </si>
+  <si>
+    <t>Entire homes &amp; apartments</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -267,6 +287,27 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -303,10 +344,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
@@ -320,8 +362,18 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -657,12 +709,12 @@
   <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.81640625" customWidth="1"/>
-    <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="3" width="39.08984375" customWidth="1"/>
-    <col min="4" max="4" width="30.36328125" customWidth="1"/>
-    <col min="6" max="6" width="26.54296875" customWidth="1"/>
-    <col min="7" max="7" width="22.36328125" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="22.81640625"/>
+    <col min="2" max="2" customWidth="true" width="36.0"/>
+    <col min="3" max="3" customWidth="true" width="39.08984375"/>
+    <col min="4" max="4" customWidth="true" width="30.36328125"/>
+    <col min="6" max="6" customWidth="true" width="26.54296875"/>
+    <col min="7" max="7" customWidth="true" width="22.36328125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -691,12 +743,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:8" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>2</v>
@@ -708,22 +760,22 @@
         <v>5</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="G2" s="1"/>
-      <c r="H2" t="s">
-        <v>47</v>
+      <c r="H2" t="s" s="0">
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>12</v>
       </c>
       <c r="D3" s="1">
         <v>2</v>
@@ -732,24 +784,24 @@
         <v>3</v>
       </c>
       <c r="F3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" t="s">
-        <v>47</v>
+      <c r="H3" t="s" s="0">
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="D4" s="1">
         <v>4</v>
@@ -758,24 +810,24 @@
         <v>7</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" t="s">
-        <v>47</v>
+        <v>16</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D5" s="1">
         <v>2</v>
@@ -784,24 +836,24 @@
         <v>4</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>21</v>
+        <v>74</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" t="s">
-        <v>47</v>
+        <v>19</v>
+      </c>
+      <c r="H5" t="s" s="0">
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D6" s="1">
         <v>1</v>
@@ -810,24 +862,24 @@
         <v>5</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H6" t="s">
-        <v>47</v>
+        <v>23</v>
+      </c>
+      <c r="H6" t="s" s="0">
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D7" s="1">
         <v>3</v>
@@ -836,22 +888,24 @@
         <v>2</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H7" s="4"/>
+        <v>27</v>
+      </c>
+      <c r="H7" t="s" s="0">
+        <v>42</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D8" s="1">
         <v>6</v>
@@ -860,22 +914,24 @@
         <v>10</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="H8" s="4"/>
+        <v>31</v>
+      </c>
+      <c r="H8" t="s" s="0">
+        <v>42</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D9" s="1">
         <v>2</v>
@@ -884,22 +940,24 @@
         <v>3</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="H9" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="H9" t="s" s="0">
+        <v>42</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D10" s="1">
         <v>4</v>
@@ -908,22 +966,24 @@
         <v>6</v>
       </c>
       <c r="F10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H10" t="s" s="0">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="H10" s="4"/>
-    </row>
-    <row r="11" spans="1:8" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>44</v>
       </c>
       <c r="D11" s="1">
         <v>2</v>
@@ -932,19 +992,21 @@
         <v>8</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="H11" s="4"/>
-    </row>
-    <row r="12" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>70</v>
+      </c>
+      <c r="H11" t="s" s="0">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1">
@@ -954,20 +1016,24 @@
         <v>3</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="G12" s="1"/>
-      <c r="H12" s="4"/>
+        <v>72</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H12" t="s" s="0">
+        <v>42</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D13" s="1">
         <v>2</v>
@@ -976,22 +1042,22 @@
         <v>4</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="H13" s="4"/>
     </row>
     <row r="14" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="D14" s="1">
         <v>1</v>
@@ -1000,7 +1066,7 @@
         <v>2</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="G14" s="1"/>
       <c r="H14" s="4"/>
@@ -1009,4 +1075,90 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0117331D-B10E-4247-8A8E-0A9EA2A2E12E}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" customWidth="true" width="8.6328125"/>
+    <col min="2" max="2" customWidth="true" width="21.6328125"/>
+    <col min="3" max="3" customWidth="true" width="21.0"/>
+    <col min="4" max="4" customWidth="true" width="18.453125"/>
+    <col min="5" max="5" customWidth="true" width="15.1796875"/>
+    <col min="6" max="6" customWidth="true" width="11.54296875"/>
+    <col min="7" max="7" customWidth="true" width="14.26953125"/>
+    <col min="8" max="8" customWidth="true" width="13.26953125"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="73" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" t="s" s="0">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" t="s" s="0">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{BC9A6F7B-B5AF-44A8-ABD1-BD1835C1A214}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{00F44353-79CE-4A3A-B0F7-E9D392F21737}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>